<commit_message>
Fixed General README File, Added README Files in Components3DModelling and PlatformDeck folders, Fixed 2025 BOM
</commit_message>
<xml_diff>
--- a/BOM/F1TenthBOM2025.xlsx
+++ b/BOM/F1TenthBOM2025.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28227"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/21d5a7416cd372e3/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\ROBORACER2025HARDWARE\hardware\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{087ACFAA-59F0-4FCC-B794-79E8558FEBD1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD3BEBB8-BB19-4B68-B0B9-051FF97FB7A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{E952CDEA-D455-4E88-9923-6EC0C627BA95}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="82">
   <si>
     <t>Number</t>
   </si>
@@ -249,6 +249,39 @@
   </si>
   <si>
     <t>Power LED 5mm</t>
+  </si>
+  <si>
+    <t>DM Stickers</t>
+  </si>
+  <si>
+    <t>Boost Converter and Lipo Connector</t>
+  </si>
+  <si>
+    <t>Pin Connecors</t>
+  </si>
+  <si>
+    <t>Step Down Converters</t>
+  </si>
+  <si>
+    <t>DP Adaptors</t>
+  </si>
+  <si>
+    <t>Step Up Boost Converters</t>
+  </si>
+  <si>
+    <t>Batteries</t>
+  </si>
+  <si>
+    <t>Screws</t>
+  </si>
+  <si>
+    <t>PPM Connectors</t>
+  </si>
+  <si>
+    <t>KabelBlinder</t>
+  </si>
+  <si>
+    <t>Boost Convertor and Rastclip</t>
   </si>
 </sst>
 </file>
@@ -346,10 +379,8 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -684,7 +715,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2885D97C-F218-4C29-A8A5-B8FE3BDF9188}">
-  <dimension ref="A1:G25"/>
+  <dimension ref="A1:G36"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12" bestFit="1" customWidth="1"/>
@@ -756,7 +787,7 @@
         <v>33.99</v>
       </c>
       <c r="E3" s="3">
-        <f t="shared" ref="E3:E24" si="0">D3*C3</f>
+        <f t="shared" ref="E3:E35" si="0">D3*C3</f>
         <v>33.99</v>
       </c>
       <c r="F3" s="2" t="s">
@@ -1023,7 +1054,7 @@
         <f>D14*C14</f>
         <v>5.69</v>
       </c>
-      <c r="F14" s="7" t="s">
+      <c r="F14" s="2" t="s">
         <v>37</v>
       </c>
       <c r="G14" s="2" t="s">
@@ -1047,7 +1078,7 @@
         <f t="shared" si="0"/>
         <v>6.99</v>
       </c>
-      <c r="F15" s="7" t="s">
+      <c r="F15" s="2" t="s">
         <v>48</v>
       </c>
       <c r="G15" s="2" t="s">
@@ -1071,7 +1102,7 @@
         <f t="shared" si="0"/>
         <v>4.09</v>
       </c>
-      <c r="F16" s="7" t="s">
+      <c r="F16" s="2" t="s">
         <v>50</v>
       </c>
       <c r="G16" s="2" t="s">
@@ -1082,7 +1113,7 @@
       <c r="A17" s="4">
         <v>16</v>
       </c>
-      <c r="B17" s="8" t="s">
+      <c r="B17" s="4" t="s">
         <v>53</v>
       </c>
       <c r="C17" s="4">
@@ -1095,7 +1126,7 @@
         <f t="shared" si="0"/>
         <v>3.59</v>
       </c>
-      <c r="F17" s="7" t="s">
+      <c r="F17" s="2" t="s">
         <v>54</v>
       </c>
       <c r="G17" s="2" t="s">
@@ -1106,7 +1137,7 @@
       <c r="A18" s="4">
         <v>17</v>
       </c>
-      <c r="B18" s="8" t="s">
+      <c r="B18" s="4" t="s">
         <v>57</v>
       </c>
       <c r="C18" s="4">
@@ -1119,7 +1150,7 @@
         <f t="shared" si="0"/>
         <v>5.99</v>
       </c>
-      <c r="F18" s="7" t="s">
+      <c r="F18" s="2" t="s">
         <v>37</v>
       </c>
       <c r="G18" s="2" t="s">
@@ -1130,7 +1161,7 @@
       <c r="A19" s="4">
         <v>18</v>
       </c>
-      <c r="B19" s="8" t="s">
+      <c r="B19" s="4" t="s">
         <v>59</v>
       </c>
       <c r="C19" s="4">
@@ -1143,7 +1174,7 @@
         <f t="shared" si="0"/>
         <v>7.99</v>
       </c>
-      <c r="F19" s="7" t="s">
+      <c r="F19" s="2" t="s">
         <v>60</v>
       </c>
       <c r="G19" s="2" t="s">
@@ -1154,7 +1185,7 @@
       <c r="A20" s="4">
         <v>19</v>
       </c>
-      <c r="B20" s="8" t="s">
+      <c r="B20" s="4" t="s">
         <v>63</v>
       </c>
       <c r="C20" s="4">
@@ -1167,7 +1198,7 @@
         <f t="shared" si="0"/>
         <v>8.36</v>
       </c>
-      <c r="F20" s="7" t="s">
+      <c r="F20" s="2" t="s">
         <v>54</v>
       </c>
       <c r="G20" s="2" t="s">
@@ -1178,7 +1209,7 @@
       <c r="A21" s="4">
         <v>20</v>
       </c>
-      <c r="B21" s="8" t="s">
+      <c r="B21" s="4" t="s">
         <v>65</v>
       </c>
       <c r="C21" s="4">
@@ -1191,7 +1222,7 @@
         <f t="shared" si="0"/>
         <v>6.91</v>
       </c>
-      <c r="F21" s="7" t="s">
+      <c r="F21" s="2" t="s">
         <v>60</v>
       </c>
       <c r="G21" s="2" t="s">
@@ -1202,7 +1233,7 @@
       <c r="A22" s="4">
         <v>21</v>
       </c>
-      <c r="B22" s="8" t="s">
+      <c r="B22" s="4" t="s">
         <v>67</v>
       </c>
       <c r="C22" s="4">
@@ -1215,7 +1246,7 @@
         <f t="shared" si="0"/>
         <v>8.58</v>
       </c>
-      <c r="F22" s="7" t="s">
+      <c r="F22" s="2" t="s">
         <v>54</v>
       </c>
       <c r="G22" s="2" t="s">
@@ -1226,7 +1257,7 @@
       <c r="A23" s="4">
         <v>22</v>
       </c>
-      <c r="B23" s="8" t="s">
+      <c r="B23" s="4" t="s">
         <v>70</v>
       </c>
       <c r="C23" s="4">
@@ -1239,7 +1270,7 @@
         <f t="shared" si="0"/>
         <v>5.99</v>
       </c>
-      <c r="F23" s="7" t="s">
+      <c r="F23" s="2" t="s">
         <v>60</v>
       </c>
       <c r="G23" s="2" t="s">
@@ -1250,7 +1281,7 @@
       <c r="A24" s="4">
         <v>23</v>
       </c>
-      <c r="B24" s="8" t="s">
+      <c r="B24" s="4" t="s">
         <v>61</v>
       </c>
       <c r="C24" s="4">
@@ -1263,7 +1294,7 @@
         <f t="shared" si="0"/>
         <v>38.950000000000003</v>
       </c>
-      <c r="F24" s="7" t="s">
+      <c r="F24" s="2" t="s">
         <v>60</v>
       </c>
       <c r="G24" s="2" t="s">
@@ -1271,12 +1302,232 @@
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="D25" s="5" t="s">
+      <c r="A25" s="4">
+        <v>24</v>
+      </c>
+      <c r="B25" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="C25" s="4">
+        <v>1</v>
+      </c>
+      <c r="D25" s="3">
+        <v>37.1</v>
+      </c>
+      <c r="E25" s="3">
+        <f t="shared" si="0"/>
+        <v>37.1</v>
+      </c>
+      <c r="F25" s="8"/>
+      <c r="G25" s="8"/>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A26" s="4">
+        <v>25</v>
+      </c>
+      <c r="B26" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="C26" s="4">
+        <v>1</v>
+      </c>
+      <c r="D26" s="3">
+        <v>19.98</v>
+      </c>
+      <c r="E26" s="3">
+        <f t="shared" si="0"/>
+        <v>19.98</v>
+      </c>
+      <c r="F26" s="8"/>
+      <c r="G26" s="8"/>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A27" s="4">
+        <v>26</v>
+      </c>
+      <c r="B27" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="C27" s="4">
+        <v>1</v>
+      </c>
+      <c r="D27" s="3">
+        <v>8.99</v>
+      </c>
+      <c r="E27" s="3">
+        <f t="shared" si="0"/>
+        <v>8.99</v>
+      </c>
+      <c r="F27" s="8"/>
+      <c r="G27" s="8"/>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A28" s="4">
+        <v>27</v>
+      </c>
+      <c r="B28" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="C28" s="4">
+        <v>1</v>
+      </c>
+      <c r="D28" s="3">
+        <v>10.79</v>
+      </c>
+      <c r="E28" s="7">
+        <f t="shared" si="0"/>
+        <v>10.79</v>
+      </c>
+      <c r="F28" s="8"/>
+      <c r="G28" s="8"/>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A29" s="4">
+        <v>28</v>
+      </c>
+      <c r="B29" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="C29" s="4">
+        <v>1</v>
+      </c>
+      <c r="D29" s="3">
+        <v>11.88</v>
+      </c>
+      <c r="E29" s="7">
+        <f t="shared" si="0"/>
+        <v>11.88</v>
+      </c>
+      <c r="F29" s="8"/>
+      <c r="G29" s="8"/>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A30" s="4">
+        <v>29</v>
+      </c>
+      <c r="B30" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="C30" s="4">
+        <v>1</v>
+      </c>
+      <c r="D30" s="3">
+        <v>7.99</v>
+      </c>
+      <c r="E30" s="7">
+        <f t="shared" si="0"/>
+        <v>7.99</v>
+      </c>
+      <c r="F30" s="8"/>
+      <c r="G30" s="8"/>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A31" s="4">
+        <v>30</v>
+      </c>
+      <c r="B31" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="C31" s="4">
+        <v>1</v>
+      </c>
+      <c r="D31" s="3">
+        <v>205.98</v>
+      </c>
+      <c r="E31" s="7">
+        <f t="shared" si="0"/>
+        <v>205.98</v>
+      </c>
+      <c r="F31" s="8"/>
+      <c r="G31" s="8"/>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A32" s="4">
+        <v>31</v>
+      </c>
+      <c r="B32" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="C32" s="4">
+        <v>1</v>
+      </c>
+      <c r="D32" s="3">
+        <v>12</v>
+      </c>
+      <c r="E32" s="7">
+        <f t="shared" si="0"/>
+        <v>12</v>
+      </c>
+      <c r="F32" s="8"/>
+      <c r="G32" s="8"/>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A33" s="4">
+        <v>32</v>
+      </c>
+      <c r="B33" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="C33" s="4">
+        <v>1</v>
+      </c>
+      <c r="D33" s="3">
+        <v>4</v>
+      </c>
+      <c r="E33" s="7">
+        <f t="shared" si="0"/>
+        <v>4</v>
+      </c>
+      <c r="F33" s="8"/>
+      <c r="G33" s="8"/>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A34" s="4">
+        <v>33</v>
+      </c>
+      <c r="B34" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="C34" s="4">
+        <v>1</v>
+      </c>
+      <c r="D34" s="3">
+        <v>13</v>
+      </c>
+      <c r="E34" s="7">
+        <f t="shared" si="0"/>
+        <v>13</v>
+      </c>
+      <c r="F34" s="8"/>
+      <c r="G34" s="8"/>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A35" s="4">
+        <v>34</v>
+      </c>
+      <c r="B35" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="C35" s="4">
+        <v>1</v>
+      </c>
+      <c r="D35" s="3">
+        <v>24.4</v>
+      </c>
+      <c r="E35" s="7">
+        <f t="shared" si="0"/>
+        <v>24.4</v>
+      </c>
+      <c r="F35" s="8"/>
+      <c r="G35" s="8"/>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="D36" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="E25" s="6">
-        <f>SUM(E2:E13)</f>
-        <v>3232.1099999999997</v>
+      <c r="E36" s="6">
+        <f>SUM(E2:E35)</f>
+        <v>3691.3499999999985</v>
       </c>
     </row>
   </sheetData>

</xml_diff>